<commit_message>
feat: improved webpage (#1)
* combine pack start and starts

* fix hurdles cells

* improved things
</commit_message>
<xml_diff>
--- a/DunbarLayout.xlsx
+++ b/DunbarLayout.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/stevenbarlow/Documents/Athletics/Markings/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/stevenbarlow/code/rydeAthletics/markings/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1B2BB44-1ECC-A147-8FAD-25C75F6F5D83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE5B0174-E7D0-4F40-A526-6180BFF6D745}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20" yWindow="680" windowWidth="29400" windowHeight="17340" xr2:uid="{E8AB9068-D317-4044-92F0-9148BCE181C7}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="29400" windowHeight="17340" xr2:uid="{E8AB9068-D317-4044-92F0-9148BCE181C7}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan" sheetId="8" r:id="rId1"/>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="512" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="512" uniqueCount="84">
   <si>
     <t>X</t>
   </si>
@@ -311,6 +311,9 @@
   </si>
   <si>
     <t>Manually Entered (Based on 3000m offsets)</t>
+  </si>
+  <si>
+    <t>H-3-3</t>
   </si>
 </sst>
 </file>
@@ -5307,7 +5310,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{D4D21C8C-4550-C84B-91F5-843380875269}" type="CELLRANGE">
+                    <a:fld id="{8DC4BDFF-FB6A-604A-8373-D29B98B5183A}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -5339,7 +5342,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{9A77649F-9129-FE49-8944-196A7CBFE403}" type="CELLRANGE">
+                    <a:fld id="{720E5872-3295-5D45-A69F-D3026C3AD0C9}" type="CELLRANGE">
                       <a:rPr lang="en-GB"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -5372,7 +5375,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{3EEE9F26-D67C-D041-9CA1-2E84FFB954EE}" type="CELLRANGE">
+                    <a:fld id="{56A95304-188D-3948-96C7-2AA9B0A53C5A}" type="CELLRANGE">
                       <a:rPr lang="en-GB"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -5405,7 +5408,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{C2031E23-EDF7-2444-A97F-B1F857EC5915}" type="CELLRANGE">
+                    <a:fld id="{BE3B9D91-61AD-B540-8427-63511E4DA587}" type="CELLRANGE">
                       <a:rPr lang="en-GB"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -5438,7 +5441,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{A0108B92-E2E9-BE42-A7D3-478D2DDC14A9}" type="CELLRANGE">
+                    <a:fld id="{7045F69A-542C-D449-A1CC-0D405EEFFFA9}" type="CELLRANGE">
                       <a:rPr lang="en-GB"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -5471,7 +5474,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{ED889AD6-3C42-F947-A24C-022F5592E8E1}" type="CELLRANGE">
+                    <a:fld id="{2EA3ABE9-A12C-0240-A567-D39B1CEE72FF}" type="CELLRANGE">
                       <a:rPr lang="en-GB"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -5504,7 +5507,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{AB27BB80-F97F-8142-8543-F37A3E50BA37}" type="CELLRANGE">
+                    <a:fld id="{62ADDF93-CFD5-654B-88D2-7357F31C8BC6}" type="CELLRANGE">
                       <a:rPr lang="en-GB"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -5537,7 +5540,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{647F00C3-9CCA-5146-9CFF-0EBD5CFF5C39}" type="CELLRANGE">
+                    <a:fld id="{237083D9-665A-B34E-AD92-1FD417022357}" type="CELLRANGE">
                       <a:rPr lang="en-GB"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -5570,7 +5573,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{E6FB0027-C2E7-EC40-AB43-1DF904354BAA}" type="CELLRANGE">
+                    <a:fld id="{434158FF-0A2F-CF4C-BA6D-D91899FC1F72}" type="CELLRANGE">
                       <a:rPr lang="en-GB"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -5603,7 +5606,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{AEFDB63B-BFDA-5944-B4BA-01D6C5DD2047}" type="CELLRANGE">
+                    <a:fld id="{63090BC9-C39A-6D4E-910F-4CFC218573D7}" type="CELLRANGE">
                       <a:rPr lang="en-GB"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -5636,7 +5639,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{9D4025C1-001D-5F40-8FDF-2DED473BA4EB}" type="CELLRANGE">
+                    <a:fld id="{5D317C30-D6DD-D540-A319-804CDC166CF4}" type="CELLRANGE">
                       <a:rPr lang="en-GB"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -5669,7 +5672,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{92E44D20-7109-B442-8DDB-F13E1D04A73D}" type="CELLRANGE">
+                    <a:fld id="{509CE872-7EE3-2F45-9FE9-2DF41AB71739}" type="CELLRANGE">
                       <a:rPr lang="en-GB"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -5702,7 +5705,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{FBC41DCB-DEBB-5C4C-8F57-7EA98EB1BB4D}" type="CELLRANGE">
+                    <a:fld id="{ADECF9B2-05ED-2D47-A9FB-7E4EAA3897FB}" type="CELLRANGE">
                       <a:rPr lang="en-GB"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -5735,7 +5738,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{CC35C747-7DF9-AD4A-89E4-145E8249A549}" type="CELLRANGE">
+                    <a:fld id="{9CE3ECEF-6625-6F4F-B52C-5AE1EA3F69DF}" type="CELLRANGE">
                       <a:rPr lang="en-GB"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -5768,7 +5771,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{D6CB8591-E391-F44E-AB73-E3C76B93CA29}" type="CELLRANGE">
+                    <a:fld id="{A56E5C08-4FAB-9941-A9FF-3BC90AA38388}" type="CELLRANGE">
                       <a:rPr lang="en-GB"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -5801,7 +5804,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{7F1F59CE-A7AB-CA4F-A341-5218780D8278}" type="CELLRANGE">
+                    <a:fld id="{46C1D3D6-F148-2A47-9DA7-9C9D91D4B640}" type="CELLRANGE">
                       <a:rPr lang="en-GB"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -5834,7 +5837,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{3B78752F-D2C2-8949-9A5B-56B311CC1B22}" type="CELLRANGE">
+                    <a:fld id="{3048942E-5566-E04D-84EE-22D959210FB4}" type="CELLRANGE">
                       <a:rPr lang="en-GB"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -5867,7 +5870,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{FDC6F91B-682D-DB44-9D0B-71C4AEFFF223}" type="CELLRANGE">
+                    <a:fld id="{ACCF54C0-CA22-F742-9660-B5E1AFFF6B91}" type="CELLRANGE">
                       <a:rPr lang="en-GB"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -5900,7 +5903,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{53EFBB64-7FF3-9E4C-99E0-10BD9B6A96C7}" type="CELLRANGE">
+                    <a:fld id="{08D9F3E8-70B8-C04D-A0FE-C5E95925E628}" type="CELLRANGE">
                       <a:rPr lang="en-GB"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -5933,7 +5936,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{E901A295-8D56-1E40-B8A4-F43BBDF8DF5B}" type="CELLRANGE">
+                    <a:fld id="{8EC6A544-4A60-EA4E-B485-CF1EFDC07B03}" type="CELLRANGE">
                       <a:rPr lang="en-GB"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -5966,7 +5969,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{CF61254D-5E37-214D-8AA2-C4A03B87F55D}" type="CELLRANGE">
+                    <a:fld id="{3AFBF3E7-E814-2940-9DAA-AB6DE41F97E2}" type="CELLRANGE">
                       <a:rPr lang="en-GB"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -9137,7 +9140,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{14E94B45-F188-A44D-AD81-C9023905F660}" type="CELLRANGE">
+                    <a:fld id="{8FEDF7F9-8DEA-E34D-BAE0-833C206D1887}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -9250,7 +9253,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>76.89</c:v>
+                  <c:v>77.336183184677466</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -9265,7 +9268,7 @@
                   <c:v>-38.99</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-38.99</c:v>
+                  <c:v>41.42759733035107</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -9278,7 +9281,7 @@
                 <c15:dlblRangeCache>
                   <c:ptCount val="1"/>
                   <c:pt idx="0">
-                    <c:v>76.89</c:v>
+                    <c:v>111.57</c:v>
                   </c:pt>
                 </c15:dlblRangeCache>
               </c15:datalabelsRange>
@@ -10536,15 +10539,15 @@
         <v>75</v>
       </c>
       <c r="T4" s="40" t="s">
-        <v>5</v>
+        <v>83</v>
       </c>
       <c r="U4" s="44">
         <f>IFERROR(VLOOKUP(T4,AllPoints,2,FALSE),0)</f>
-        <v>76.89</v>
+        <v>77.336183184677466</v>
       </c>
       <c r="V4" s="45">
         <f>IFERROR(VLOOKUP(T4,AllPoints,3,FALSE),0)</f>
-        <v>-38.99</v>
+        <v>41.42759733035107</v>
       </c>
     </row>
     <row r="5" spans="19:22" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -10553,15 +10556,15 @@
       </c>
       <c r="T5" s="41">
         <f>SQRT((U4-U3)^2+(V4-V3)^2)</f>
-        <v>76.89</v>
+        <v>111.57004611436027</v>
       </c>
       <c r="U5" s="44">
         <f>ABS(U4-U3)</f>
-        <v>76.89</v>
+        <v>77.336183184677466</v>
       </c>
       <c r="V5" s="45">
         <f>ABS(V4-V3)</f>
-        <v>0</v>
+        <v>80.417597330351072</v>
       </c>
     </row>
     <row r="15" spans="19:22" x14ac:dyDescent="0.2">

</xml_diff>